<commit_message>
updating MYA price to september WASDE
</commit_message>
<xml_diff>
--- a/data-raw/fsaArcPlc/input_data/fsaMyaPrice/MYA_2025.xlsx
+++ b/data-raw/fsaArcPlc/input_data/fsaMyaPrice/MYA_2025.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28925"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\EPAS\2014FBIMP\ARC_PLC\Webpage Posting\2025-0812\Program Year 2025\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\EPAS\2014FBIMP\ARC_PLC\Webpage Posting\2025-0912\Program Year 2025\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA8EE359-F884-41C2-B254-8DB6502E0F01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0EF5ACC1-3FB8-4483-9D0E-6AAE978EA7C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
     <t>TABLE 1. 2019/20-2025/26 MARKET YEAR AVERAGE (MYA) PRICES</t>
   </si>
   <si>
-    <t>August 12, 2025 1/</t>
+    <t>September 12, 2025 1/</t>
   </si>
   <si>
     <t>Commodity</t>
@@ -691,7 +691,7 @@
         <v>17</v>
       </c>
       <c r="L5" s="6">
-        <v>5.3</v>
+        <v>5.0999999999999996</v>
       </c>
       <c r="M5" s="7" t="s">
         <v>18</v>
@@ -808,10 +808,10 @@
         <v>0.26900000000000002</v>
       </c>
       <c r="J8" s="8">
-        <v>0.25900000000000001</v>
+        <v>0.26100000000000001</v>
       </c>
       <c r="K8" s="7" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L8" s="9">
         <v>0.25</v>
@@ -937,7 +937,7 @@
         <v>18</v>
       </c>
       <c r="L11" s="6">
-        <v>10.1</v>
+        <v>10</v>
       </c>
       <c r="M11" s="7" t="s">
         <v>18</v>
@@ -978,7 +978,7 @@
         <v>17</v>
       </c>
       <c r="L12" s="9">
-        <v>0.151</v>
+        <v>0.13700000000000001</v>
       </c>
       <c r="M12" s="7" t="s">
         <v>18</v>
@@ -1019,7 +1019,7 @@
         <v>17</v>
       </c>
       <c r="L13" s="9">
-        <v>0.40600000000000003</v>
+        <v>0.38400000000000001</v>
       </c>
       <c r="M13" s="7" t="s">
         <v>18</v>
@@ -1060,7 +1060,7 @@
         <v>17</v>
       </c>
       <c r="L14" s="9">
-        <v>0.21</v>
+        <v>0.22</v>
       </c>
       <c r="M14" s="7" t="s">
         <v>18</v>
@@ -1095,13 +1095,13 @@
         <v>0.36899999999999999</v>
       </c>
       <c r="J15" s="8">
-        <v>0.33900000000000002</v>
+        <v>0.34399999999999997</v>
       </c>
       <c r="K15" s="7" t="s">
         <v>18</v>
       </c>
       <c r="L15" s="9">
-        <v>0.29499999999999998</v>
+        <v>0.33300000000000002</v>
       </c>
       <c r="M15" s="7" t="s">
         <v>18</v>
@@ -1136,13 +1136,13 @@
         <v>0.35699999999999998</v>
       </c>
       <c r="J16" s="8">
-        <v>0.26400000000000001</v>
+        <v>0.26</v>
       </c>
       <c r="K16" s="7" t="s">
         <v>18</v>
       </c>
       <c r="L16" s="9">
-        <v>0.317</v>
+        <v>0.30099999999999999</v>
       </c>
       <c r="M16" s="7" t="s">
         <v>18</v>
@@ -1183,7 +1183,7 @@
         <v>18</v>
       </c>
       <c r="L17" s="9">
-        <v>0.22600000000000001</v>
+        <v>0.23050000000000001</v>
       </c>
       <c r="M17" s="7" t="s">
         <v>18</v>
@@ -1224,7 +1224,7 @@
         <v>17</v>
       </c>
       <c r="L18" s="9">
-        <v>12.8</v>
+        <v>13.5</v>
       </c>
       <c r="M18" s="7" t="s">
         <v>18</v>
@@ -1470,7 +1470,7 @@
         <v>18</v>
       </c>
       <c r="L24" s="9">
-        <v>0.34189999999999998</v>
+        <v>0.34250000000000003</v>
       </c>
       <c r="M24" s="7" t="s">
         <v>18</v>
@@ -1505,13 +1505,13 @@
         <v>0.159</v>
       </c>
       <c r="J25" s="8">
-        <v>0.14099999999999999</v>
+        <v>0.14000000000000001</v>
       </c>
       <c r="K25" s="7" t="s">
         <v>18</v>
       </c>
       <c r="L25" s="9">
-        <v>0.13</v>
+        <v>0.12</v>
       </c>
       <c r="M25" s="7" t="s">
         <v>18</v>
@@ -1552,7 +1552,7 @@
         <v>18</v>
       </c>
       <c r="L26" s="9">
-        <v>0.13500000000000001</v>
+        <v>0.125</v>
       </c>
       <c r="M26" s="7" t="s">
         <v>18</v>
@@ -1593,7 +1593,7 @@
         <v>18</v>
       </c>
       <c r="L27" s="13">
-        <v>0.21</v>
+        <v>0.2</v>
       </c>
       <c r="M27" s="14" t="s">
         <v>18</v>

</xml_diff>

<commit_message>
updating 2025 mya prices
</commit_message>
<xml_diff>
--- a/data-raw/fsaArcPlc/input_data/fsaMyaPrice/MYA_2025.xlsx
+++ b/data-raw/fsaArcPlc/input_data/fsaMyaPrice/MYA_2025.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29231"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\EPAS\2014FBIMP\ARC_PLC\Webpage Posting\2025-0912\Program Year 2025\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\EPAS\2014FBIMP\ARC_PLC\Webpage Posting\2025-1114\Program Year 2025\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0EF5ACC1-3FB8-4483-9D0E-6AAE978EA7C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FC7DD66-458F-49F6-8480-16DBDBAD6031}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="MYA Prices" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0" concurrentCalc="0"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
@@ -25,7 +25,7 @@
     <t>TABLE 1. 2019/20-2025/26 MARKET YEAR AVERAGE (MYA) PRICES</t>
   </si>
   <si>
-    <t>September 12, 2025 1/</t>
+    <t>November 14, 2025 1/</t>
   </si>
   <si>
     <t>Commodity</t>
@@ -573,19 +573,19 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:M32"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="12" customHeight="1" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="12" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="22.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="10" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="2.140625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="2.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="22.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.88671875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="10" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="2.109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="2.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:13" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="15" t="s">
         <v>0</v>
       </c>
@@ -602,7 +602,7 @@
       <c r="L1" s="16"/>
       <c r="M1" s="16"/>
     </row>
-    <row r="2" spans="1:13" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:13" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="15" t="s">
         <v>1</v>
       </c>
@@ -619,7 +619,7 @@
       <c r="L2" s="16"/>
       <c r="M2" s="16"/>
     </row>
-    <row r="4" spans="1:13" ht="65.099999999999994" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:13" ht="64.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>2</v>
       </c>
@@ -656,7 +656,7 @@
       </c>
       <c r="M4" s="19"/>
     </row>
-    <row r="5" spans="1:13" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:13" ht="13.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>13</v>
       </c>
@@ -691,13 +691,13 @@
         <v>17</v>
       </c>
       <c r="L5" s="6">
-        <v>5.0999999999999996</v>
+        <v>5</v>
       </c>
       <c r="M5" s="7" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:13" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:13" ht="13.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
         <v>19</v>
       </c>
@@ -738,7 +738,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="7" spans="1:13" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:13" ht="13.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
         <v>20</v>
       </c>
@@ -779,7 +779,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="8" spans="1:13" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:13" ht="13.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
         <v>21</v>
       </c>
@@ -820,7 +820,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="9" spans="1:13" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:13" ht="13.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
         <v>25</v>
       </c>
@@ -849,19 +849,19 @@
         <v>4.55</v>
       </c>
       <c r="J9" s="5">
-        <v>4.3</v>
+        <v>4.24</v>
       </c>
       <c r="K9" s="7" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L9" s="6">
-        <v>3.9</v>
+        <v>4</v>
       </c>
       <c r="M9" s="7" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="10" spans="1:13" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:13" ht="13.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
         <v>28</v>
       </c>
@@ -890,19 +890,19 @@
         <v>4.93</v>
       </c>
       <c r="J10" s="5">
-        <v>4.0999999999999996</v>
+        <v>4.07</v>
       </c>
       <c r="K10" s="7" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L10" s="6">
-        <v>3.7</v>
+        <v>3.8</v>
       </c>
       <c r="M10" s="7" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="11" spans="1:13" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:13" ht="13.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
         <v>29</v>
       </c>
@@ -934,16 +934,16 @@
         <v>10</v>
       </c>
       <c r="K11" s="7" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L11" s="6">
-        <v>10</v>
+        <v>10.5</v>
       </c>
       <c r="M11" s="7" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="12" spans="1:13" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:13" ht="13.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
         <v>30</v>
       </c>
@@ -978,13 +978,13 @@
         <v>17</v>
       </c>
       <c r="L12" s="9">
-        <v>0.13700000000000001</v>
+        <v>0.11799999999999999</v>
       </c>
       <c r="M12" s="7" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="13" spans="1:13" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:13" ht="13.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="3" t="s">
         <v>33</v>
       </c>
@@ -1019,13 +1019,13 @@
         <v>17</v>
       </c>
       <c r="L13" s="9">
-        <v>0.38400000000000001</v>
+        <v>0.313</v>
       </c>
       <c r="M13" s="7" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="14" spans="1:13" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:13" ht="13.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="3" t="s">
         <v>34</v>
       </c>
@@ -1060,13 +1060,13 @@
         <v>17</v>
       </c>
       <c r="L14" s="9">
-        <v>0.22</v>
+        <v>0.215</v>
       </c>
       <c r="M14" s="7" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="15" spans="1:13" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:13" ht="13.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="3" t="s">
         <v>35</v>
       </c>
@@ -1095,19 +1095,19 @@
         <v>0.36899999999999999</v>
       </c>
       <c r="J15" s="8">
-        <v>0.34399999999999997</v>
+        <v>0.34300000000000003</v>
       </c>
       <c r="K15" s="7" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L15" s="9">
-        <v>0.33300000000000002</v>
+        <v>0.28000000000000003</v>
       </c>
       <c r="M15" s="7" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="16" spans="1:13" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:13" ht="13.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="3" t="s">
         <v>36</v>
       </c>
@@ -1136,19 +1136,19 @@
         <v>0.35699999999999998</v>
       </c>
       <c r="J16" s="8">
-        <v>0.26</v>
+        <v>0.25600000000000001</v>
       </c>
       <c r="K16" s="7" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L16" s="9">
-        <v>0.30099999999999999</v>
+        <v>0.19400000000000001</v>
       </c>
       <c r="M16" s="7" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="17" spans="1:13" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:13" ht="13.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="3" t="s">
         <v>37</v>
       </c>
@@ -1177,10 +1177,10 @@
         <v>0.21199999999999999</v>
       </c>
       <c r="J17" s="8">
-        <v>0.23300000000000001</v>
+        <v>0.23799999999999999</v>
       </c>
       <c r="K17" s="7" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L17" s="9">
         <v>0.23050000000000001</v>
@@ -1189,7 +1189,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="18" spans="1:13" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:13" ht="13.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="3" t="s">
         <v>38</v>
       </c>
@@ -1230,7 +1230,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="19" spans="1:13" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:13" ht="13.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="3" t="s">
         <v>39</v>
       </c>
@@ -1259,19 +1259,19 @@
         <v>0.57899999999999996</v>
       </c>
       <c r="J19" s="8">
-        <v>0.45</v>
+        <v>0.44900000000000001</v>
       </c>
       <c r="K19" s="7" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L19" s="9">
-        <v>0.41</v>
+        <v>0.42799999999999999</v>
       </c>
       <c r="M19" s="7" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="20" spans="1:13" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:13" ht="13.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="3" t="s">
         <v>40</v>
       </c>
@@ -1306,13 +1306,13 @@
         <v>17</v>
       </c>
       <c r="L20" s="9">
-        <v>0.3</v>
+        <v>0.3125</v>
       </c>
       <c r="M20" s="7" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="21" spans="1:13" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:13" ht="13.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="3" t="s">
         <v>41</v>
       </c>
@@ -1344,16 +1344,16 @@
         <v>0.24299999999999999</v>
       </c>
       <c r="K21" s="7" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L21" s="9">
-        <v>0.22</v>
+        <v>0.23</v>
       </c>
       <c r="M21" s="7" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="22" spans="1:13" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:13" ht="13.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="3" t="s">
         <v>42</v>
       </c>
@@ -1385,16 +1385,16 @@
         <v>0.39400000000000002</v>
       </c>
       <c r="K22" s="7" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L22" s="9">
-        <v>0.36</v>
+        <v>0.375</v>
       </c>
       <c r="M22" s="7" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="23" spans="1:13" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:13" ht="13.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="3" t="s">
         <v>43</v>
       </c>
@@ -1423,10 +1423,10 @@
         <v>0.4</v>
       </c>
       <c r="J23" s="8">
-        <v>0.39</v>
+        <v>0.54</v>
       </c>
       <c r="K23" s="7" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L23" s="9">
         <v>0.33</v>
@@ -1435,7 +1435,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="24" spans="1:13" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:13" ht="13.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="3" t="s">
         <v>44</v>
       </c>
@@ -1464,19 +1464,19 @@
         <v>0.39489999999999997</v>
       </c>
       <c r="J24" s="8">
-        <v>0.34010000000000001</v>
+        <v>0.34039999999999998</v>
       </c>
       <c r="K24" s="7" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L24" s="9">
-        <v>0.34250000000000003</v>
+        <v>0.3337</v>
       </c>
       <c r="M24" s="7" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="25" spans="1:13" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:13" ht="13.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="3" t="s">
         <v>45</v>
       </c>
@@ -1511,13 +1511,13 @@
         <v>18</v>
       </c>
       <c r="L25" s="9">
-        <v>0.12</v>
+        <v>0.115</v>
       </c>
       <c r="M25" s="7" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="26" spans="1:13" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:13" ht="13.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="3" t="s">
         <v>47</v>
       </c>
@@ -1552,13 +1552,13 @@
         <v>18</v>
       </c>
       <c r="L26" s="9">
-        <v>0.125</v>
+        <v>0.12</v>
       </c>
       <c r="M26" s="7" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="27" spans="1:13" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:13" ht="13.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="10" t="s">
         <v>48</v>
       </c>
@@ -1599,7 +1599,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="29" spans="1:13" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:13" ht="13.05" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="17" t="s">
         <v>51</v>
       </c>
@@ -1616,7 +1616,7 @@
       <c r="L29" s="17"/>
       <c r="M29" s="17"/>
     </row>
-    <row r="30" spans="1:13" ht="26.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:13" ht="25.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="17" t="s">
         <v>52</v>
       </c>
@@ -1633,7 +1633,7 @@
       <c r="L30" s="17"/>
       <c r="M30" s="17"/>
     </row>
-    <row r="31" spans="1:13" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:13" ht="13.05" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="17" t="s">
         <v>53</v>
       </c>
@@ -1650,7 +1650,7 @@
       <c r="L31" s="17"/>
       <c r="M31" s="17"/>
     </row>
-    <row r="32" spans="1:13" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:13" ht="13.05" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="17" t="s">
         <v>54</v>
       </c>

</xml_diff>

<commit_message>
Update MYA 2025 Excel and related data files
Refreshed MYA_2025.xlsx and regenerated fsaArcPlcData.rda and fsaMyaPrice.rda to reflect updated MYA price data for 2025.
</commit_message>
<xml_diff>
--- a/data-raw/fsaArcPlc/input_data/fsaMyaPrice/MYA_2025.xlsx
+++ b/data-raw/fsaArcPlc/input_data/fsaMyaPrice/MYA_2025.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29328"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\EPAS\2014FBIMP\ARC_PLC\Webpage Posting\2025-1114\Program Year 2025\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\EPAS\2014FBIMP\ARC_PLC\Webpage Posting\2025-1215\Program Year 2025\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FC7DD66-458F-49F6-8480-16DBDBAD6031}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1BC68A4F-693E-4BCD-BEE0-312933C848E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="MYA Prices" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="0" concurrentCalc="0"/>
 </workbook>
 </file>
 
@@ -25,7 +25,7 @@
     <t>TABLE 1. 2019/20-2025/26 MARKET YEAR AVERAGE (MYA) PRICES</t>
   </si>
   <si>
-    <t>November 14, 2025 1/</t>
+    <t>December 15, 2025 1/</t>
   </si>
   <si>
     <t>Commodity</t>
@@ -573,19 +573,19 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:M32"/>
-  <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="12" customHeight="1" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="12" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="22.88671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.88671875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.44140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="10" width="11.109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="2.109375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.109375" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="2.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="22.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="10" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="2.140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="2.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="15" t="s">
         <v>0</v>
       </c>
@@ -602,7 +602,7 @@
       <c r="L1" s="16"/>
       <c r="M1" s="16"/>
     </row>
-    <row r="2" spans="1:13" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:13" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="15" t="s">
         <v>1</v>
       </c>
@@ -619,7 +619,7 @@
       <c r="L2" s="16"/>
       <c r="M2" s="16"/>
     </row>
-    <row r="4" spans="1:13" ht="64.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:13" ht="65.099999999999994" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>2</v>
       </c>
@@ -656,7 +656,7 @@
       </c>
       <c r="M4" s="19"/>
     </row>
-    <row r="5" spans="1:13" ht="13.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:13" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
         <v>13</v>
       </c>
@@ -697,7 +697,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:13" ht="13.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:13" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="3" t="s">
         <v>19</v>
       </c>
@@ -738,7 +738,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="7" spans="1:13" ht="13.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:13" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="3" t="s">
         <v>20</v>
       </c>
@@ -779,7 +779,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="8" spans="1:13" ht="13.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:13" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="3" t="s">
         <v>21</v>
       </c>
@@ -820,7 +820,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="9" spans="1:13" ht="13.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:13" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="3" t="s">
         <v>25</v>
       </c>
@@ -861,7 +861,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="10" spans="1:13" ht="13.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:13" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="3" t="s">
         <v>28</v>
       </c>
@@ -902,7 +902,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="11" spans="1:13" ht="13.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:13" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="3" t="s">
         <v>29</v>
       </c>
@@ -943,7 +943,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="12" spans="1:13" ht="13.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:13" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="3" t="s">
         <v>30</v>
       </c>
@@ -984,7 +984,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="13" spans="1:13" ht="13.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:13" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="3" t="s">
         <v>33</v>
       </c>
@@ -1025,7 +1025,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="14" spans="1:13" ht="13.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:13" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="3" t="s">
         <v>34</v>
       </c>
@@ -1066,7 +1066,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="15" spans="1:13" ht="13.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:13" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="3" t="s">
         <v>35</v>
       </c>
@@ -1107,7 +1107,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="16" spans="1:13" ht="13.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:13" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="3" t="s">
         <v>36</v>
       </c>
@@ -1148,7 +1148,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="17" spans="1:13" ht="13.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:13" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="3" t="s">
         <v>37</v>
       </c>
@@ -1189,7 +1189,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="18" spans="1:13" ht="13.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:13" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="3" t="s">
         <v>38</v>
       </c>
@@ -1230,7 +1230,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="19" spans="1:13" ht="13.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:13" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="3" t="s">
         <v>39</v>
       </c>
@@ -1271,7 +1271,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="20" spans="1:13" ht="13.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:13" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="3" t="s">
         <v>40</v>
       </c>
@@ -1312,7 +1312,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="21" spans="1:13" ht="13.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:13" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="3" t="s">
         <v>41</v>
       </c>
@@ -1353,7 +1353,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="22" spans="1:13" ht="13.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:13" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="3" t="s">
         <v>42</v>
       </c>
@@ -1394,7 +1394,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="23" spans="1:13" ht="13.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:13" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="3" t="s">
         <v>43</v>
       </c>
@@ -1435,7 +1435,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="24" spans="1:13" ht="13.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:13" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="3" t="s">
         <v>44</v>
       </c>
@@ -1470,13 +1470,13 @@
         <v>17</v>
       </c>
       <c r="L24" s="9">
-        <v>0.3337</v>
+        <v>0.32519999999999999</v>
       </c>
       <c r="M24" s="7" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="25" spans="1:13" ht="13.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:13" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="3" t="s">
         <v>45</v>
       </c>
@@ -1508,16 +1508,16 @@
         <v>0.14000000000000001</v>
       </c>
       <c r="K25" s="7" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L25" s="9">
-        <v>0.115</v>
+        <v>0.105</v>
       </c>
       <c r="M25" s="7" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="26" spans="1:13" ht="13.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:13" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="3" t="s">
         <v>47</v>
       </c>
@@ -1546,19 +1546,19 @@
         <v>0.17199999999999999</v>
       </c>
       <c r="J26" s="8">
-        <v>0.152</v>
+        <v>0.15</v>
       </c>
       <c r="K26" s="7" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L26" s="9">
-        <v>0.12</v>
+        <v>0.11</v>
       </c>
       <c r="M26" s="7" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="27" spans="1:13" ht="13.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:13" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="10" t="s">
         <v>48</v>
       </c>
@@ -1593,13 +1593,13 @@
         <v>18</v>
       </c>
       <c r="L27" s="13">
-        <v>0.2</v>
+        <v>0.18</v>
       </c>
       <c r="M27" s="14" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="29" spans="1:13" ht="13.05" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:13" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="17" t="s">
         <v>51</v>
       </c>
@@ -1616,7 +1616,7 @@
       <c r="L29" s="17"/>
       <c r="M29" s="17"/>
     </row>
-    <row r="30" spans="1:13" ht="25.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:13" ht="26.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="17" t="s">
         <v>52</v>
       </c>
@@ -1633,7 +1633,7 @@
       <c r="L30" s="17"/>
       <c r="M30" s="17"/>
     </row>
-    <row r="31" spans="1:13" ht="13.05" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:13" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="17" t="s">
         <v>53</v>
       </c>
@@ -1650,7 +1650,7 @@
       <c r="L31" s="17"/>
       <c r="M31" s="17"/>
     </row>
-    <row r="32" spans="1:13" ht="13.05" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:13" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="17" t="s">
         <v>54</v>
       </c>

</xml_diff>

<commit_message>
updating mya prices, arc co benchmarks, and acreage
updating mya prices, arc co benchmarks, and acreage
</commit_message>
<xml_diff>
--- a/data-raw/fsaArcPlc/input_data/fsaMyaPrice/MYA_2025.xlsx
+++ b/data-raw/fsaArcPlc/input_data/fsaMyaPrice/MYA_2025.xlsx
@@ -1,31 +1,31 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29426"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\EPAS\2014FBIMP\ARC_PLC\Webpage Posting\2025-1215\Program Year 2025\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\EPAS\2014FBIMP\ARC_PLC\Webpage Posting\2026-0130\Program Year 2025\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1BC68A4F-693E-4BCD-BEE0-312933C848E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29F2D654-05E3-4151-914B-A57D4A1A8E46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="MYA Prices" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0" concurrentCalc="0"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="56">
   <si>
     <t>TABLE 1. 2019/20-2025/26 MARKET YEAR AVERAGE (MYA) PRICES</t>
   </si>
   <si>
-    <t>December 15, 2025 1/</t>
+    <t>January 30, 2026 1/</t>
   </si>
   <si>
     <t>Commodity</t>
@@ -119,6 +119,9 @@
   </si>
   <si>
     <t>July 31, 2026</t>
+  </si>
+  <si>
+    <t>.</t>
   </si>
   <si>
     <t>Lentils</t>
@@ -573,19 +576,19 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:M32"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="12" customHeight="1" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="12" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="22.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="10" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="2.140625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="2.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="22.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.88671875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="10" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="2.109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="2.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:13" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="15" t="s">
         <v>0</v>
       </c>
@@ -602,7 +605,7 @@
       <c r="L1" s="16"/>
       <c r="M1" s="16"/>
     </row>
-    <row r="2" spans="1:13" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:13" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="15" t="s">
         <v>1</v>
       </c>
@@ -619,7 +622,7 @@
       <c r="L2" s="16"/>
       <c r="M2" s="16"/>
     </row>
-    <row r="4" spans="1:13" ht="65.099999999999994" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:13" ht="64.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>2</v>
       </c>
@@ -656,7 +659,7 @@
       </c>
       <c r="M4" s="19"/>
     </row>
-    <row r="5" spans="1:13" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:13" ht="13.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>13</v>
       </c>
@@ -691,13 +694,13 @@
         <v>17</v>
       </c>
       <c r="L5" s="6">
-        <v>5</v>
+        <v>4.9000000000000004</v>
       </c>
       <c r="M5" s="7" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:13" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:13" ht="13.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
         <v>19</v>
       </c>
@@ -732,13 +735,13 @@
         <v>17</v>
       </c>
       <c r="L6" s="6">
-        <v>5.3</v>
+        <v>5.4</v>
       </c>
       <c r="M6" s="7" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="7" spans="1:13" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:13" ht="13.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
         <v>20</v>
       </c>
@@ -773,13 +776,13 @@
         <v>17</v>
       </c>
       <c r="L7" s="6">
-        <v>3.1</v>
+        <v>3.15</v>
       </c>
       <c r="M7" s="7" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="8" spans="1:13" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:13" ht="13.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
         <v>21</v>
       </c>
@@ -814,13 +817,13 @@
         <v>17</v>
       </c>
       <c r="L8" s="9">
-        <v>0.25</v>
+        <v>0.245</v>
       </c>
       <c r="M8" s="7" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="9" spans="1:13" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:13" ht="13.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
         <v>25</v>
       </c>
@@ -855,13 +858,13 @@
         <v>17</v>
       </c>
       <c r="L9" s="6">
-        <v>4</v>
+        <v>4.0999999999999996</v>
       </c>
       <c r="M9" s="7" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="10" spans="1:13" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:13" ht="13.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
         <v>28</v>
       </c>
@@ -896,13 +899,13 @@
         <v>17</v>
       </c>
       <c r="L10" s="6">
-        <v>3.8</v>
+        <v>3.7</v>
       </c>
       <c r="M10" s="7" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="11" spans="1:13" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:13" ht="13.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
         <v>29</v>
       </c>
@@ -937,13 +940,13 @@
         <v>17</v>
       </c>
       <c r="L11" s="6">
-        <v>10.5</v>
+        <v>10.199999999999999</v>
       </c>
       <c r="M11" s="7" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="12" spans="1:13" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:13" ht="13.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
         <v>30</v>
       </c>
@@ -977,16 +980,16 @@
       <c r="K12" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="L12" s="9">
-        <v>0.11799999999999999</v>
+      <c r="L12" s="9" t="s">
+        <v>33</v>
       </c>
       <c r="M12" s="7" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="13" spans="1:13" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:13" ht="13.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="3" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B13" s="4" t="s">
         <v>31</v>
@@ -1018,16 +1021,16 @@
       <c r="K13" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="L13" s="9">
-        <v>0.313</v>
+      <c r="L13" s="9" t="s">
+        <v>33</v>
       </c>
       <c r="M13" s="7" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="14" spans="1:13" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:13" ht="13.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B14" s="4" t="s">
         <v>31</v>
@@ -1060,15 +1063,15 @@
         <v>17</v>
       </c>
       <c r="L14" s="9">
-        <v>0.215</v>
+        <v>0.20499999999999999</v>
       </c>
       <c r="M14" s="7" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="15" spans="1:13" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:13" ht="13.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="3" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B15" s="4" t="s">
         <v>26</v>
@@ -1100,16 +1103,16 @@
       <c r="K15" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="L15" s="9">
-        <v>0.28000000000000003</v>
+      <c r="L15" s="9" t="s">
+        <v>33</v>
       </c>
       <c r="M15" s="7" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="16" spans="1:13" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:13" ht="13.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="3" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B16" s="4" t="s">
         <v>26</v>
@@ -1141,16 +1144,16 @@
       <c r="K16" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="L16" s="9">
-        <v>0.19400000000000001</v>
+      <c r="L16" s="9" t="s">
+        <v>33</v>
       </c>
       <c r="M16" s="7" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="17" spans="1:13" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:13" ht="13.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="3" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B17" s="4" t="s">
         <v>26</v>
@@ -1183,15 +1186,15 @@
         <v>17</v>
       </c>
       <c r="L17" s="9">
-        <v>0.23050000000000001</v>
+        <v>0.22850000000000001</v>
       </c>
       <c r="M17" s="7" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="18" spans="1:13" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:13" ht="13.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="3" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B18" s="4" t="s">
         <v>31</v>
@@ -1224,15 +1227,15 @@
         <v>17</v>
       </c>
       <c r="L18" s="9">
-        <v>13.5</v>
+        <v>13</v>
       </c>
       <c r="M18" s="7" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="19" spans="1:13" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:13" ht="13.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="3" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B19" s="4" t="s">
         <v>26</v>
@@ -1265,15 +1268,15 @@
         <v>17</v>
       </c>
       <c r="L19" s="9">
-        <v>0.42799999999999999</v>
+        <v>0.41</v>
       </c>
       <c r="M19" s="7" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="20" spans="1:13" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:13" ht="13.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="3" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B20" s="4" t="s">
         <v>31</v>
@@ -1306,15 +1309,15 @@
         <v>17</v>
       </c>
       <c r="L20" s="9">
-        <v>0.3125</v>
+        <v>0.3</v>
       </c>
       <c r="M20" s="7" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="21" spans="1:13" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:13" ht="13.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="3" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B21" s="4" t="s">
         <v>26</v>
@@ -1347,15 +1350,15 @@
         <v>17</v>
       </c>
       <c r="L21" s="9">
-        <v>0.23</v>
+        <v>0.215</v>
       </c>
       <c r="M21" s="7" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="22" spans="1:13" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:13" ht="13.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="3" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B22" s="4" t="s">
         <v>26</v>
@@ -1388,15 +1391,15 @@
         <v>17</v>
       </c>
       <c r="L22" s="9">
-        <v>0.375</v>
+        <v>0.36</v>
       </c>
       <c r="M22" s="7" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="23" spans="1:13" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:13" ht="13.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="3" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B23" s="4" t="s">
         <v>26</v>
@@ -1435,9 +1438,9 @@
         <v>18</v>
       </c>
     </row>
-    <row r="24" spans="1:13" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:13" ht="13.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B24" s="4" t="s">
         <v>22</v>
@@ -1470,21 +1473,21 @@
         <v>17</v>
       </c>
       <c r="L24" s="9">
-        <v>0.32519999999999999</v>
+        <v>0.33350000000000002</v>
       </c>
       <c r="M24" s="7" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="25" spans="1:13" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:13" ht="13.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B25" s="4" t="s">
         <v>22</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D25" s="4" t="s">
         <v>24</v>
@@ -1517,15 +1520,15 @@
         <v>18</v>
       </c>
     </row>
-    <row r="26" spans="1:13" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:13" ht="13.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="3" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B26" s="4" t="s">
         <v>22</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D26" s="4" t="s">
         <v>24</v>
@@ -1552,21 +1555,21 @@
         <v>17</v>
       </c>
       <c r="L26" s="9">
-        <v>0.11</v>
+        <v>0.13500000000000001</v>
       </c>
       <c r="M26" s="7" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="27" spans="1:13" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:13" ht="13.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="10" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B27" s="11" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C27" s="11" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D27" s="11" t="s">
         <v>24</v>
@@ -1587,10 +1590,10 @@
         <v>0.223</v>
       </c>
       <c r="J27" s="12">
-        <v>0.2</v>
+        <v>0.187</v>
       </c>
       <c r="K27" s="14" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L27" s="13">
         <v>0.18</v>
@@ -1599,9 +1602,9 @@
         <v>18</v>
       </c>
     </row>
-    <row r="29" spans="1:13" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:13" ht="13.05" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="17" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B29" s="17"/>
       <c r="C29" s="17"/>
@@ -1616,9 +1619,9 @@
       <c r="L29" s="17"/>
       <c r="M29" s="17"/>
     </row>
-    <row r="30" spans="1:13" ht="26.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:13" ht="25.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="17" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B30" s="17"/>
       <c r="C30" s="17"/>
@@ -1633,9 +1636,9 @@
       <c r="L30" s="17"/>
       <c r="M30" s="17"/>
     </row>
-    <row r="31" spans="1:13" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:13" ht="13.05" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="17" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B31" s="17"/>
       <c r="C31" s="17"/>
@@ -1650,9 +1653,9 @@
       <c r="L31" s="17"/>
       <c r="M31" s="17"/>
     </row>
-    <row r="32" spans="1:13" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:13" ht="13.05" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="17" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B32" s="17"/>
       <c r="C32" s="17"/>

</xml_diff>

<commit_message>
updating mya price and arc plc data based on latest wasde
</commit_message>
<xml_diff>
--- a/data-raw/fsaArcPlc/input_data/fsaMyaPrice/MYA_2025.xlsx
+++ b/data-raw/fsaArcPlc/input_data/fsaMyaPrice/MYA_2025.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\EPAS\2014FBIMP\ARC_PLC\Webpage Posting\2026-0210\Program Year 2025\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\EPAS\2014FBIMP\ARC_PLC\Webpage Posting\2026-0310\Program Year 2025\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3AD5359B-8AE7-4CC2-B8C0-7ED628C0B03A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA5683E0-A52C-4AAB-A85A-E2E5132E71F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-15120" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="MYA Prices" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
     <t>TABLE 1. 2019/20-2025/26 MARKET YEAR AVERAGE (MYA) PRICES</t>
   </si>
   <si>
-    <t>February 10, 2026 1/</t>
+    <t>March 10, 2026 1/</t>
   </si>
   <si>
     <t>Commodity</t>
@@ -203,16 +203,19 @@
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="8"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="4">
@@ -689,7 +692,7 @@
         <v>5.52</v>
       </c>
       <c r="K5" s="6">
-        <v>4.9000000000000004</v>
+        <v>4.95</v>
       </c>
       <c r="L5" s="8" t="s">
         <v>17</v>
@@ -727,7 +730,7 @@
         <v>6.31</v>
       </c>
       <c r="K6" s="6">
-        <v>5.4</v>
+        <v>5.45</v>
       </c>
       <c r="L6" s="8" t="s">
         <v>17</v>
@@ -803,7 +806,7 @@
         <v>0.26100000000000001</v>
       </c>
       <c r="K8" s="10">
-        <v>0.24</v>
+        <v>0.23499999999999999</v>
       </c>
       <c r="L8" s="8" t="s">
         <v>17</v>
@@ -879,7 +882,7 @@
         <v>4.07</v>
       </c>
       <c r="K10" s="6">
-        <v>3.6</v>
+        <v>3.55</v>
       </c>
       <c r="L10" s="8" t="s">
         <v>17</v>
@@ -955,7 +958,7 @@
         <v>0.13600000000000001</v>
       </c>
       <c r="K12" s="10">
-        <v>0.108</v>
+        <v>0.11799999999999999</v>
       </c>
       <c r="L12" s="8" t="s">
         <v>17</v>
@@ -993,7 +996,7 @@
         <v>0.35899999999999999</v>
       </c>
       <c r="K13" s="10">
-        <v>0.247</v>
+        <v>0.22800000000000001</v>
       </c>
       <c r="L13" s="8" t="s">
         <v>17</v>
@@ -1069,7 +1072,7 @@
         <v>0.34300000000000003</v>
       </c>
       <c r="K15" s="10">
-        <v>0.32</v>
+        <v>0.28000000000000003</v>
       </c>
       <c r="L15" s="8" t="s">
         <v>17</v>
@@ -1107,7 +1110,7 @@
         <v>0.25600000000000001</v>
       </c>
       <c r="K16" s="10">
-        <v>0.20499999999999999</v>
+        <v>0.17100000000000001</v>
       </c>
       <c r="L16" s="8" t="s">
         <v>17</v>
@@ -1145,7 +1148,7 @@
         <v>0.23799999999999999</v>
       </c>
       <c r="K17" s="10">
-        <v>0.22850000000000001</v>
+        <v>0.22700000000000001</v>
       </c>
       <c r="L17" s="8" t="s">
         <v>17</v>
@@ -1183,7 +1186,7 @@
         <v>12.5</v>
       </c>
       <c r="K18" s="10">
-        <v>13</v>
+        <v>12.75</v>
       </c>
       <c r="L18" s="8" t="s">
         <v>17</v>
@@ -1221,7 +1224,7 @@
         <v>0.44900000000000001</v>
       </c>
       <c r="K19" s="10">
-        <v>0.41</v>
+        <v>0.3085</v>
       </c>
       <c r="L19" s="8" t="s">
         <v>17</v>
@@ -1259,7 +1262,7 @@
         <v>0.32800000000000001</v>
       </c>
       <c r="K20" s="10">
-        <v>0.3</v>
+        <v>0.26700000000000002</v>
       </c>
       <c r="L20" s="8" t="s">
         <v>17</v>
@@ -1297,7 +1300,7 @@
         <v>0.24299999999999999</v>
       </c>
       <c r="K21" s="10">
-        <v>0.215</v>
+        <v>0.20300000000000001</v>
       </c>
       <c r="L21" s="8" t="s">
         <v>17</v>
@@ -1335,7 +1338,7 @@
         <v>0.39400000000000002</v>
       </c>
       <c r="K22" s="10">
-        <v>0.36</v>
+        <v>0.32</v>
       </c>
       <c r="L22" s="8" t="s">
         <v>17</v>
@@ -1411,7 +1414,7 @@
         <v>0.34039999999999998</v>
       </c>
       <c r="K24" s="10">
-        <v>0.32919999999999999</v>
+        <v>0.3291</v>
       </c>
       <c r="L24" s="8" t="s">
         <v>17</v>
@@ -1487,7 +1490,7 @@
         <v>0.15</v>
       </c>
       <c r="K26" s="10">
-        <v>0.13800000000000001</v>
+        <v>0.14199999999999999</v>
       </c>
       <c r="L26" s="8" t="s">
         <v>17</v>

</xml_diff>

<commit_message>
updating mya prices, arc co benchmarks, and enrolled base
</commit_message>
<xml_diff>
--- a/data-raw/fsaArcPlc/input_data/fsaMyaPrice/MYA_2025.xlsx
+++ b/data-raw/fsaArcPlc/input_data/fsaMyaPrice/MYA_2025.xlsx
@@ -1,31 +1,31 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30131"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\EPAS\2014FBIMP\ARC_PLC\Webpage Posting\2026-0520\Program Year 2025\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\EPAS\2014FBIMP\ARC_PLC\Webpage Posting\2026-0812\Program Year 2025\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDB660C0-06DE-4B22-A999-48DBDD8FC6D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F207D484-727D-40B7-88F6-CF1C8B086BC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="MYA Prices" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0" concurrentCalc="0"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="55">
   <si>
     <t>TABLE 1. 2019/20-2025/26 MARKET YEAR AVERAGE (MYA) PRICES</t>
   </si>
   <si>
-    <t>May 20, 2026 1/</t>
+    <t>August 12, 2026 1/</t>
   </si>
   <si>
     <t>Commodity</t>
@@ -73,25 +73,28 @@
     <t>Bushel</t>
   </si>
   <si>
+    <t>F</t>
+  </si>
+  <si>
+    <t>Barley</t>
+  </si>
+  <si>
+    <t>Oats</t>
+  </si>
+  <si>
+    <t>Peanuts</t>
+  </si>
+  <si>
+    <t>Aug. 1-Jul. 31</t>
+  </si>
+  <si>
+    <t>August 31, 2026</t>
+  </si>
+  <si>
+    <t>Pound</t>
+  </si>
+  <si>
     <t>P</t>
-  </si>
-  <si>
-    <t>Barley</t>
-  </si>
-  <si>
-    <t>Oats</t>
-  </si>
-  <si>
-    <t>Peanuts</t>
-  </si>
-  <si>
-    <t>Aug. 1-Jul. 31</t>
-  </si>
-  <si>
-    <t>August 31, 2026</t>
-  </si>
-  <si>
-    <t>Pound</t>
   </si>
   <si>
     <t>Corn</t>
@@ -203,19 +206,16 @@
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
       <sz val="8"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="4">
@@ -692,7 +692,7 @@
         <v>5.52</v>
       </c>
       <c r="K5" s="6">
-        <v>5</v>
+        <v>5.0599999999999996</v>
       </c>
       <c r="L5" s="8" t="s">
         <v>17</v>
@@ -730,7 +730,7 @@
         <v>6.31</v>
       </c>
       <c r="K6" s="6">
-        <v>5.45</v>
+        <v>5.46</v>
       </c>
       <c r="L6" s="8" t="s">
         <v>17</v>
@@ -768,7 +768,7 @@
         <v>3.35</v>
       </c>
       <c r="K7" s="6">
-        <v>3.25</v>
+        <v>3.23</v>
       </c>
       <c r="L7" s="8" t="s">
         <v>17</v>
@@ -806,21 +806,21 @@
         <v>0.26100000000000001</v>
       </c>
       <c r="K8" s="10">
-        <v>0.23300000000000001</v>
+        <v>0.23599999999999999</v>
       </c>
       <c r="L8" s="8" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
     </row>
     <row r="9" spans="1:12" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="3" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D9" s="4" t="s">
         <v>16</v>
@@ -847,18 +847,18 @@
         <v>4.1500000000000004</v>
       </c>
       <c r="L9" s="8" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
     </row>
     <row r="10" spans="1:12" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C10" s="4" t="s">
         <v>27</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>26</v>
       </c>
       <c r="D10" s="4" t="s">
         <v>16</v>
@@ -885,18 +885,18 @@
         <v>3.55</v>
       </c>
       <c r="L10" s="8" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
     </row>
     <row r="11" spans="1:12" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D11" s="4" t="s">
         <v>16</v>
@@ -923,18 +923,18 @@
         <v>10.4</v>
       </c>
       <c r="L11" s="8" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
     </row>
     <row r="12" spans="1:12" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="3" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D12" s="4" t="s">
         <v>23</v>
@@ -958,7 +958,7 @@
         <v>0.13600000000000001</v>
       </c>
       <c r="K12" s="10">
-        <v>0.113</v>
+        <v>0.111</v>
       </c>
       <c r="L12" s="8" t="s">
         <v>17</v>
@@ -966,13 +966,13 @@
     </row>
     <row r="13" spans="1:12" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C13" s="4" t="s">
         <v>32</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="C13" s="4" t="s">
-        <v>31</v>
       </c>
       <c r="D13" s="4" t="s">
         <v>23</v>
@@ -996,7 +996,7 @@
         <v>0.35899999999999999</v>
       </c>
       <c r="K13" s="10">
-        <v>0.22700000000000001</v>
+        <v>0.22</v>
       </c>
       <c r="L13" s="8" t="s">
         <v>17</v>
@@ -1004,13 +1004,13 @@
     </row>
     <row r="14" spans="1:12" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="3" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D14" s="4" t="s">
         <v>23</v>
@@ -1034,7 +1034,7 @@
         <v>0.20200000000000001</v>
       </c>
       <c r="K14" s="10">
-        <v>0.20799999999999999</v>
+        <v>0.21099999999999999</v>
       </c>
       <c r="L14" s="8" t="s">
         <v>17</v>
@@ -1042,13 +1042,13 @@
     </row>
     <row r="15" spans="1:12" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D15" s="4" t="s">
         <v>23</v>
@@ -1072,21 +1072,21 @@
         <v>0.34300000000000003</v>
       </c>
       <c r="K15" s="10">
-        <v>0.247</v>
+        <v>0.25600000000000001</v>
       </c>
       <c r="L15" s="8" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
     </row>
     <row r="16" spans="1:12" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="3" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D16" s="4" t="s">
         <v>23</v>
@@ -1110,21 +1110,21 @@
         <v>0.25600000000000001</v>
       </c>
       <c r="K16" s="10">
-        <v>0.16200000000000001</v>
+        <v>0.16300000000000001</v>
       </c>
       <c r="L16" s="8" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
     </row>
     <row r="17" spans="1:12" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="3" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D17" s="4" t="s">
         <v>23</v>
@@ -1148,21 +1148,21 @@
         <v>0.23799999999999999</v>
       </c>
       <c r="K17" s="10">
-        <v>0.24049999999999999</v>
+        <v>0.23499999999999999</v>
       </c>
       <c r="L17" s="8" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
     </row>
     <row r="18" spans="1:12" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="3" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D18" s="4" t="s">
         <v>16</v>
@@ -1186,7 +1186,7 @@
         <v>12.5</v>
       </c>
       <c r="K18" s="10">
-        <v>12.65</v>
+        <v>12.6</v>
       </c>
       <c r="L18" s="8" t="s">
         <v>17</v>
@@ -1194,13 +1194,13 @@
     </row>
     <row r="19" spans="1:12" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="3" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D19" s="4" t="s">
         <v>23</v>
@@ -1224,21 +1224,21 @@
         <v>0.44900000000000001</v>
       </c>
       <c r="K19" s="10">
-        <v>0.313</v>
+        <v>0.3075</v>
       </c>
       <c r="L19" s="8" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
     </row>
     <row r="20" spans="1:12" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="3" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D20" s="4" t="s">
         <v>23</v>
@@ -1270,13 +1270,13 @@
     </row>
     <row r="21" spans="1:12" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="3" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D21" s="4" t="s">
         <v>23</v>
@@ -1303,18 +1303,18 @@
         <v>0.20799999999999999</v>
       </c>
       <c r="L21" s="8" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
     </row>
     <row r="22" spans="1:12" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="3" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D22" s="4" t="s">
         <v>23</v>
@@ -1341,18 +1341,18 @@
         <v>0.32</v>
       </c>
       <c r="L22" s="8" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
     </row>
     <row r="23" spans="1:12" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="3" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D23" s="4" t="s">
         <v>23</v>
@@ -1379,18 +1379,18 @@
         <v>0.33</v>
       </c>
       <c r="L23" s="8" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
     </row>
     <row r="24" spans="1:12" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="3" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B24" s="4" t="s">
         <v>21</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D24" s="4" t="s">
         <v>23</v>
@@ -1414,21 +1414,21 @@
         <v>0.34039999999999998</v>
       </c>
       <c r="K24" s="10">
-        <v>0.34549999999999997</v>
+        <v>0.33889999999999998</v>
       </c>
       <c r="L24" s="8" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
     </row>
     <row r="25" spans="1:12" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B25" s="4" t="s">
         <v>21</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D25" s="4" t="s">
         <v>23</v>
@@ -1455,18 +1455,18 @@
         <v>0.104</v>
       </c>
       <c r="L25" s="8" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
     </row>
     <row r="26" spans="1:12" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="3" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B26" s="4" t="s">
         <v>21</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D26" s="4" t="s">
         <v>23</v>
@@ -1490,21 +1490,21 @@
         <v>0.15</v>
       </c>
       <c r="K26" s="10">
-        <v>0.14699999999999999</v>
+        <v>0.14899999999999999</v>
       </c>
       <c r="L26" s="8" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
     </row>
     <row r="27" spans="1:12" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="12" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B27" s="13" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C27" s="13" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D27" s="13" t="s">
         <v>23</v>
@@ -1528,15 +1528,15 @@
         <v>0.187</v>
       </c>
       <c r="K27" s="15">
-        <v>0.20300000000000001</v>
+        <v>0.20200000000000001</v>
       </c>
       <c r="L27" s="17" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
     </row>
     <row r="29" spans="1:12" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="20" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B29" s="20"/>
       <c r="C29" s="20"/>
@@ -1552,7 +1552,7 @@
     </row>
     <row r="30" spans="1:12" ht="26.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="20" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B30" s="20"/>
       <c r="C30" s="20"/>
@@ -1568,7 +1568,7 @@
     </row>
     <row r="31" spans="1:12" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="20" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B31" s="20"/>
       <c r="C31" s="20"/>
@@ -1584,7 +1584,7 @@
     </row>
     <row r="32" spans="1:12" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="20" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B32" s="20"/>
       <c r="C32" s="20"/>

</xml_diff>